<commit_message>
[fix] Tauri 위젯 룸 컨텍스트와 Windows 실행 보강 (#164)
* [fix] 로그인 후 위젯 프로젝트룸 복구 보강

* [fix] 위젯 룸 컨텍스트와 Windows 실행 보강

* [fix] 활동 감지 실백엔드 스모크 보강

* [fix] 위젯 실행 실패 재시도 상태 보강

* [fix] 위젯 표시 데이터 서버 우선 복구

* [fix] 위젯 사용량 동기화 실패 재시도 보강

* [fix] 위젯 창 실행 안정화

* [fix] 위젯 창 안정화 범위 분리

* [fix] 위젯 음성 API 스모크 보강

* [fix] 로컬 파일 분석 실백엔드 스모크 보강

* [fix] 로컬 파일 갱신 동기화 스모크 보강

* [fix] 활동 추적 삭제 왕복 스모크 보강

* [fix] 개인정보 동의 API 계약 정렬

* [test] 윈도우 활동 감지 실캡처 검증 추가

* [test] 로컬 폴더 감시 이벤트 검증 추가

* [fix] 로컬 SQLite 진단 정보 보강

* [fix] 활동 추적 종료 전 동기화 보강

* [test] 타이머 실백엔드 스모크 보강

* [test] 위젯 항목 상태 실백엔드 검증 보강

* [fix] 위젯 요약 캐시 계정 경계 보강

* [fix] 위젯 항목 상태 실제 아이템 경로 연결

* [fix] 위젯 항목 상태 화면 반영 보강

* [fix] 위젯 항목 상태 재조회 반영
</commit_message>
<xml_diff>
--- a/docs/tauri-widget-platform-split-checklist-2026-07-03.xlsx
+++ b/docs/tauri-widget-platform-split-checklist-2026-07-03.xlsx
@@ -51,7 +51,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +83,46 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009FD3FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008FD59D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -110,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,6 +176,58 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -675,12 +767,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>주의</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Mac 수정 병합 후 Windows에서만 재검증. 앞으로 Windows 작업 중 macOS 전용 로직은 건드리지 않는 방향.</t>
+          <t>최근 갱신</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-03 Windows: widget item controls work with real item UUIDs, apply successful state changes immediately, and reload persisted item states from /api/widget/items/states; real-backend smoke verifies state-id and task-id PATCH, item-state readback, timer lifecycle, activity/current-app, local-file sync/analysis, privacy consent, widget usage, and account-partitioned widget summary cache. macOS app/widget logic remains Mac-team owned and untouched.</t>
         </is>
       </c>
     </row>
@@ -698,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -781,7 +873,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="17" t="n">
         <v>70</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -831,7 +923,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="17" t="n">
         <v>75</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -878,35 +970,35 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>74</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>bar+todo 표시, 나머지는 바 복원 항목 시드(#162)</t>
+          <t>Login opens bar + primary widget after auth; Windows/non-mac widget open command now returns after actual Tauri window creation instead of delayed background spawn.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Mac 수정 병합 후 Windows 실사용 확인</t>
+          <t>Real OAuth Windows GUI relaunch/minimize/close/flicker regression QA remains.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>로그인 후 bar/todo 표시, 각 위젯 복원</t>
+          <t>cargo fmt/check/tests, real-backend smoke, and PR CI; GUI capture still required.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>#162</t>
+          <t>#164, authenticated-surfaces.ts, src-tauri/src/lib.rs</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>창 다중 오픈/깜빡임 재발 확인</t>
+          <t>macOS keeps the previous async widget build path; Mac team owns Mac widget fix.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -928,35 +1020,35 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>72</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>열기/닫기/최소화/복원/항상 위/고스트/위치 저장</t>
+          <t>Open/close/minimize/restore/topmost/ghost/position store; Windows/non-mac existing windows now reapply saved preferred-monitor position and close-all/context persist immediately.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>투명창, 무테두리, 그림자 GUI QA</t>
+          <t>Transparent frameless shadow and no-scrollbar GUI capture QA.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>창 테두리 없음, 스크롤바 없음, 드래그 가능</t>
+          <t>cargo test --lib; actual Windows Tauri screen capture must show no border/scrollbar/titlebar flicker.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>src-tauri/src/lib.rs, desktop-widget</t>
+          <t>#164, src-tauri/src/lib.rs, desktop-widget</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Windows WebView shadow/transparent 확인</t>
+          <t>Windows WebView transparent/shadow QA still required; macOS async build path preserved.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -976,40 +1068,40 @@
           <t>SQLite</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>꽤 됨</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>bundled rusqlite, auth/room/folder/file/FTS/outbox/widget/activity/timer/cache/backup</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>실앱 장시간 DB 무결성/복구 QA</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>quick_check, 백업/복구, 재시작 유지</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>local_db.rs</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>현재 단위테스트 기준만 강함</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>86</v>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Bundled rusqlite, WAL, auth/room/folder/file/FTS/outbox/widget/activity/timer/cache/backup. Widget summary cache is now partitioned by current auth subject so stale seed/other-account widget data is not reused after real login. SQLite integrity IPC returns quick_check, journal mode, page/free counts, DB size, and WAL size.</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Installed-app long-run DB growth/recovery QA, restore-from-backup relaunch proof, and real-account cache rollover GUI QA remain.</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_db::tests::widget_summary_cache_is_partitioned_by_cache_key; full cargo test --lib; npm.cmd run dev:widget:backend verifies real summary path remains green.</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/local_db.rs, src/lib/widget/widget-summary-client.ts, src/lib/tauri/commands.ts</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>Common SQLite/cache contract only; macOS window/runtime logic remains Mac-team owned and untouched.</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
@@ -1026,90 +1118,90 @@
           <t>로컬 폴더 트래킹</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>폴더 등록, scan, native watch, FTS 검색, 미리보기, 열기, reindex</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>대용량/삭제/권한/장시간 watch QA</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>생성/수정/삭제가 local_file_events에 반영</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>local_files.rs</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Windows notify 경로 확인</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>74</v>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Folder register/scan/native watch/FTS/preview/open/reindex. Direct watch callback test now verifies CREATED -&gt; UPDATED -&gt; DELETED plus FTS add/remove on Windows checkout.</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Real Tauri GUI long-run watch QA, large file/permission-denied cases, and SQLite row inspection in an installed app profile.</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_files::tests::watch_path_change_records_create_update_and_delete; full cargo test --lib; real-backend local file smoke.</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/local_files.rs, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>Windows evidence only; macOS FSEvents/app-widget logic remains Mac-team owned and untouched.</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>로컬 파일 서버 동기화</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>승인 이벤트를 /api/local-file-events/sync로 전송</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>localEventId 매칭 PR #158 머지와 실백엔드 왕복</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>sync 후 올바른 이벤트가 SYNCED/FAILED</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>#158</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>현재 체크아웃에는 #158 미포함</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Approved local file CREATED/UPDATED/DELETED sync is smoke-tested. Created PERSONAL resource then posts extracted text/key sentences to /api/local-file-analyses to create an ANALYZE_RESOURCE job.</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>GUI watch/outbox long-run QA, SQLite row state inspection, and large/permission-denied file cases still remain.</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend checks /api/local-file-events/sync CREATED/UPDATED/DELETED plus /api/local-file-analyses before cleanup.</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>#164, scripts/dev-widget-real-backend.mjs, managed-folder-client.ts, localFileAnalysisApi.ts</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Windows-only verification scope; macOS widget/app path remains Mac-team owned.</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
@@ -1128,35 +1220,35 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>60</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>65</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Win32 foreground window/process 감지, 동의 기반 30초 자동 캡처</t>
+          <t>Win32 capture path remains; activity buffer resend now preserves consent and smoke records /api/activity/current-app.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>실사용 dwell time 검증</t>
+          <t>Real Tauri foreground-window dwell QA and long-run retry behavior still remain.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>앱 전환 시 appName/windowTitle 기록, /api/activity/today 반영</t>
+          <t>dev:widget:backend records smoke activity and verifies /api/activity/today contains it.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>activity.rs, activity-client.ts</t>
+          <t>#164, activity-client.ts, scripts/dev-widget-real-backend.mjs</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Windows 전용 로직 유지</t>
+          <t>Do not touch macOS activity cfg; Mac team owns macOS widget/app fix.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1178,35 +1270,35 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>75</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>90</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>로컬 상세 이벤트, rollup, 서버 usage summary 동기화</t>
+          <t>Widget display uses server-first summary fallback; usage rollups mark failed/mismatched sync attempts in SQLite for retry; desktop widget item buttons call /api/widget/items/{id}/state with real item UUID fallback, then reload persisted item states through /api/widget/items/states so CONFIRMED/HIDDEN/SNOOZED/PINNED survives refresh/reopen instead of only the current click session.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>실서버 settings 매칭 실패 케이스 QA</t>
+          <t>Manual Windows GUI QA still remains for visual click feedback and backend-side filtering once item-state-aware domain lists are expanded beyond widget state lookup.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>위젯 조작 후 rollup sync</t>
+          <t>npm.cmd run dev:widget:backend verifies state-id PATCH, task-id fallback PATCH, /api/widget/items/states readback, and DB persistence; npm.cmd run typecheck verifies frontend state application.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>widget_usage.rs</t>
+          <t>#164 frontend, backend #183, desktop-widget/page.tsx, widgetApi.ts, dev-widget-real-backend.mjs, WidgetService.java, WidgetItemStateResponse.java</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>장시간 동기화 확인</t>
+          <t>Windows/Tauri widget behavior plus backend widget API; macOS app/widget runtime remains Mac-team owned and untouched.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -1228,35 +1320,35 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>72</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>채팅방/메시지 API, 전송, 읽음, 로컬 메시지 캐시, LiveKit 진입 코드</t>
+          <t>Chat rooms/messages/read cache plus voice room create/read/mic/leave are connected in the real-backend widget smoke; widget voice type now accepts createdByUserId.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>실채팅/음성 연결 QA</t>
+          <t>LiveKit in-app audio GUI/mic permission QA and token-backed room join still need live desktop verification.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>메시지 전송/읽음/캐시, 음성방 토큰</t>
+          <t>npm.cmd run dev:widget:backend verifies chat and voice HTTP roundtrips; GUI voice join still required.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>desktop-widget/page.tsx</t>
+          <t>#164, scripts/dev-widget-real-backend.mjs, widgetDisplayApi.ts, desktop-widget/page.tsx</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>마이크 권한 확인</t>
+          <t>Token smoke is optional when local LiveKit secret is unavailable; Mac-specific logic untouched.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1281,7 +1373,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="17" t="n">
         <v>75</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1331,7 +1423,7 @@
           <t>대기</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="26" t="n">
         <v>50</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1381,7 +1473,7 @@
           <t>대기</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="26" t="n">
         <v>60</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1431,7 +1523,7 @@
           <t>문제</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="26" t="n">
         <v>30</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1481,7 +1573,7 @@
           <t>대기</t>
         </is>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="26" t="n">
         <v>40</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1531,7 +1623,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="17" t="n">
         <v>70</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1581,7 +1673,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="26" t="n">
         <v>60</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1631,7 +1723,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="26" t="n">
         <v>55</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1681,7 +1773,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="26" t="n">
         <v>55</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1731,7 +1823,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="26" t="n">
         <v>65</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1781,7 +1873,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="26" t="n">
         <v>55</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1831,7 +1923,7 @@
           <t>검증필요</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="26" t="n">
         <v>65</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1862,6 +1954,106 @@
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>Mac 팀</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>실시간 활동 추적</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>78</v>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Windows foreground app/window capture uses Win32 APIs, stores dwell in Tauri SQLite buffer, reflects consented records to /api/activity/current-app, verifies /today inclusion/delete, and now has a Windows-only real foreground capture unit test.</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>Long-running incremental capture and settings/permission UX QA in real Windows Tauri GUI remain.</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>cargo test --lib on Windows includes windows_foreground_capture_returns_app_name; npm.cmd run dev:widget:backend verifies server record/today/delete.</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/activity.rs, src/lib/local/activity-client.ts, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Windows-only test; macOS osascript/permission path is untouched and remains Mac-team owned.</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>Codex Windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Privacy consent API</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Frontend settings adapter now maps backend /api/me/privacy-consents {items:[ACTIVITY_CONTEXT, MANAGED_FOLDER]} to app booleans and PATCHes only backend-supported consent types.</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Full settings GUI toggle QA in real Tauri session remains.</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>typecheck plus npm.cmd run dev:widget:backend checks GET/PATCH /api/me/privacy-consents and managed folder re-enable before local file sync.</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>#164, settingsApi.ts, settings.ts, settings/page.tsx, privacy-consent-panel.tsx, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>Removes unsupported MANAGED_FOLDER_ACCESS/LOCAL_AGENT_MEMORY API enum usage; macOS logic untouched.</t>
+        </is>
+      </c>
+      <c r="J25" s="18" t="inlineStr">
+        <is>
+          <t>Codex Windows</t>
         </is>
       </c>
     </row>
@@ -1885,6 +2077,60 @@
     <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="2">
       <formula>60</formula>
     </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D24">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D25">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1899,7 +2145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1982,7 +2228,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="17" t="n">
         <v>70</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -2032,7 +2278,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="17" t="n">
         <v>75</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2079,35 +2325,35 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>74</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>bar+todo 표시, 나머지는 바 복원 항목 시드(#162)</t>
+          <t>Login opens bar + primary widget after auth; Windows/non-mac widget open command now returns after actual Tauri window creation instead of delayed background spawn.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Mac 수정 병합 후 Windows 실사용 확인</t>
+          <t>Real OAuth Windows GUI relaunch/minimize/close/flicker regression QA remains.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>로그인 후 bar/todo 표시, 각 위젯 복원</t>
+          <t>cargo fmt/check/tests, real-backend smoke, and PR CI; GUI capture still required.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>#162</t>
+          <t>#164, authenticated-surfaces.ts, src-tauri/src/lib.rs</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>창 다중 오픈/깜빡임 재발 확인</t>
+          <t>macOS keeps the previous async widget build path; Mac team owns Mac widget fix.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -2129,35 +2375,35 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>72</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>열기/닫기/최소화/복원/항상 위/고스트/위치 저장</t>
+          <t>Open/close/minimize/restore/topmost/ghost/position store; Windows/non-mac existing windows now reapply saved preferred-monitor position and close-all/context persist immediately.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>투명창, 무테두리, 그림자 GUI QA</t>
+          <t>Transparent frameless shadow and no-scrollbar GUI capture QA.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>창 테두리 없음, 스크롤바 없음, 드래그 가능</t>
+          <t>cargo test --lib; actual Windows Tauri screen capture must show no border/scrollbar/titlebar flicker.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>src-tauri/src/lib.rs, desktop-widget</t>
+          <t>#164, src-tauri/src/lib.rs, desktop-widget</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Windows WebView shadow/transparent 확인</t>
+          <t>Windows WebView transparent/shadow QA still required; macOS async build path preserved.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -2177,40 +2423,40 @@
           <t>SQLite</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>꽤 됨</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>bundled rusqlite, auth/room/folder/file/FTS/outbox/widget/activity/timer/cache/backup</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>실앱 장시간 DB 무결성/복구 QA</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>quick_check, 백업/복구, 재시작 유지</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>local_db.rs</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>현재 단위테스트 기준만 강함</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>86</v>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Bundled rusqlite, WAL, auth/room/folder/file/FTS/outbox/widget/activity/timer/cache/backup. Widget summary cache is now partitioned by current auth subject so stale seed/other-account widget data is not reused after real login. SQLite integrity IPC returns quick_check, journal mode, page/free counts, DB size, and WAL size.</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Installed-app long-run DB growth/recovery QA, restore-from-backup relaunch proof, and real-account cache rollover GUI QA remain.</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_db::tests::widget_summary_cache_is_partitioned_by_cache_key; full cargo test --lib; npm.cmd run dev:widget:backend verifies real summary path remains green.</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/local_db.rs, src/lib/widget/widget-summary-client.ts, src/lib/tauri/commands.ts</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>Common SQLite/cache contract only; macOS window/runtime logic remains Mac-team owned and untouched.</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
@@ -2227,90 +2473,90 @@
           <t>로컬 폴더 트래킹</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>폴더 등록, scan, native watch, FTS 검색, 미리보기, 열기, reindex</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>대용량/삭제/권한/장시간 watch QA</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>생성/수정/삭제가 local_file_events에 반영</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>local_files.rs</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Windows notify 경로 확인</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>74</v>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Folder register/scan/native watch/FTS/preview/open/reindex. Direct watch callback test now verifies CREATED -&gt; UPDATED -&gt; DELETED plus FTS add/remove on Windows checkout.</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Real Tauri GUI long-run watch QA, large file/permission-denied cases, and SQLite row inspection in an installed app profile.</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_files::tests::watch_path_change_records_create_update_and_delete; full cargo test --lib; real-backend local file smoke.</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/local_files.rs, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>Windows evidence only; macOS FSEvents/app-widget logic remains Mac-team owned and untouched.</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>로컬 파일 서버 동기화</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>승인 이벤트를 /api/local-file-events/sync로 전송</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>localEventId 매칭 PR #158 머지와 실백엔드 왕복</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>sync 후 올바른 이벤트가 SYNCED/FAILED</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>#158</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>현재 체크아웃에는 #158 미포함</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Approved local file CREATED/UPDATED/DELETED sync is smoke-tested. Created PERSONAL resource then posts extracted text/key sentences to /api/local-file-analyses to create an ANALYZE_RESOURCE job.</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>GUI watch/outbox long-run QA, SQLite row state inspection, and large/permission-denied file cases still remain.</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend checks /api/local-file-events/sync CREATED/UPDATED/DELETED plus /api/local-file-analyses before cleanup.</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>#164, scripts/dev-widget-real-backend.mjs, managed-folder-client.ts, localFileAnalysisApi.ts</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Windows-only verification scope; macOS widget/app path remains Mac-team owned.</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
@@ -2329,35 +2575,35 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>60</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>65</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Win32 foreground window/process 감지, 동의 기반 30초 자동 캡처</t>
+          <t>Win32 capture path remains; activity buffer resend now preserves consent and smoke records /api/activity/current-app.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>실사용 dwell time 검증</t>
+          <t>Real Tauri foreground-window dwell QA and long-run retry behavior still remain.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>앱 전환 시 appName/windowTitle 기록, /api/activity/today 반영</t>
+          <t>dev:widget:backend records smoke activity and verifies /api/activity/today contains it.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>activity.rs, activity-client.ts</t>
+          <t>#164, activity-client.ts, scripts/dev-widget-real-backend.mjs</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Windows 전용 로직 유지</t>
+          <t>Do not touch macOS activity cfg; Mac team owns macOS widget/app fix.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -2379,35 +2625,35 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>75</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>90</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>로컬 상세 이벤트, rollup, 서버 usage summary 동기화</t>
+          <t>Widget display uses server-first summary fallback; usage rollups mark failed/mismatched sync attempts in SQLite for retry; desktop widget item buttons call /api/widget/items/{id}/state with real item UUID fallback, then reload persisted item states through /api/widget/items/states so CONFIRMED/HIDDEN/SNOOZED/PINNED survives refresh/reopen instead of only the current click session.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>실서버 settings 매칭 실패 케이스 QA</t>
+          <t>Manual Windows GUI QA still remains for visual click feedback and backend-side filtering once item-state-aware domain lists are expanded beyond widget state lookup.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>위젯 조작 후 rollup sync</t>
+          <t>npm.cmd run dev:widget:backend verifies state-id PATCH, task-id fallback PATCH, /api/widget/items/states readback, and DB persistence; npm.cmd run typecheck verifies frontend state application.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>widget_usage.rs</t>
+          <t>#164 frontend, backend #183, desktop-widget/page.tsx, widgetApi.ts, dev-widget-real-backend.mjs, WidgetService.java, WidgetItemStateResponse.java</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>장시간 동기화 확인</t>
+          <t>Windows/Tauri widget behavior plus backend widget API; macOS app/widget runtime remains Mac-team owned and untouched.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -2429,35 +2675,35 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>진행</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>65</v>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>72</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>채팅방/메시지 API, 전송, 읽음, 로컬 메시지 캐시, LiveKit 진입 코드</t>
+          <t>Chat rooms/messages/read cache plus voice room create/read/mic/leave are connected in the real-backend widget smoke; widget voice type now accepts createdByUserId.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>실채팅/음성 연결 QA</t>
+          <t>LiveKit in-app audio GUI/mic permission QA and token-backed room join still need live desktop verification.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>메시지 전송/읽음/캐시, 음성방 토큰</t>
+          <t>npm.cmd run dev:widget:backend verifies chat and voice HTTP roundtrips; GUI voice join still required.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>desktop-widget/page.tsx</t>
+          <t>#164, scripts/dev-widget-real-backend.mjs, widgetDisplayApi.ts, desktop-widget/page.tsx</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>마이크 권한 확인</t>
+          <t>Token smoke is optional when local LiveKit secret is unavailable; Mac-specific logic untouched.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -2482,7 +2728,7 @@
           <t>진행</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="17" t="n">
         <v>75</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -2511,6 +2757,106 @@
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Codex Windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>실시간 활동 추적</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>78</v>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Windows foreground app/window capture uses Win32 APIs, stores dwell in Tauri SQLite buffer, reflects consented records to /api/activity/current-app, verifies /today inclusion/delete, and now has a Windows-only real foreground capture unit test.</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>Long-running incremental capture and settings/permission UX QA in real Windows Tauri GUI remain.</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>cargo test --lib on Windows includes windows_foreground_capture_returns_app_name; npm.cmd run dev:widget:backend verifies server record/today/delete.</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>#164, src-tauri/src/activity.rs, src/lib/local/activity-client.ts, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>Windows-only test; macOS osascript/permission path is untouched and remains Mac-team owned.</t>
+        </is>
+      </c>
+      <c r="J13" s="18" t="inlineStr">
+        <is>
+          <t>Codex Windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Privacy consent API</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>progress</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Frontend settings adapter now maps backend /api/me/privacy-consents {items:[ACTIVITY_CONTEXT, MANAGED_FOLDER]} to app booleans and PATCHes only backend-supported consent types.</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Full settings GUI toggle QA in real Tauri session remains.</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>typecheck plus npm.cmd run dev:widget:backend checks GET/PATCH /api/me/privacy-consents and managed folder re-enable before local file sync.</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>#164, settingsApi.ts, settings.ts, settings/page.tsx, privacy-consent-panel.tsx, scripts/dev-widget-real-backend.mjs</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Removes unsupported MANAGED_FOLDER_ACCESS/LOCAL_AGENT_MEMORY API enum usage; macOS logic untouched.</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
         <is>
           <t>Codex Windows</t>
         </is>
@@ -2535,6 +2881,60 @@
     </cfRule>
     <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="2">
       <formula>60</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D14">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="60"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00F4CCCC"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3201,7 +3601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3417,22 +3817,54 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>로컬 파일/활동/SQLite 실백엔드 왕복</t>
+          <t>Local file/activity/SQLite real-backend and GUI QA follow-up</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>SQLite 상태와 서버 응답 일치</t>
+          <t>API smoke passes; GUI SQLite/watch/runtime evidence captured separately</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>실백엔드 + Docker 환경</t>
+          <t>npm.cmd run dev:widget:backend + Tauri GUI QA</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>#158 병합 여부 확인</t>
+          <t>Do not modify macOS-specific logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Windows widget window runtime stabilization GUI QA</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>No delayed wave/flicker after login; preferred monitor move reapplies to visible widgets; close-all leaves no widget windows.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>npm.cmd run tauri:dev:backend + Windows screen capture; cargo test --lib</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Do not touch macOS-specific widget/app logic.</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3593,24 +4025,24 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>로컬 폴더</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>테스트 폴더 watch</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>생성/수정/삭제 반영</t>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_files::tests::watch_path_change_records_create_update_and_delete; test folder watch in Tauri GUI</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>CREATED/UPDATED/DELETED events plus FTS add/remove; GUI watch reflects created/modified/deleted files</t>
         </is>
       </c>
     </row>
@@ -3677,6 +4109,402 @@
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>생성/수정/삭제 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Real backend API smoke</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>widget, chat, local-file sync, activity, summaries pass against Docker/backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Widget launch failure retry</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Code path + typecheck + tauri-boundaries</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>All-open failure leaves launched flag false and avoids starting background runtimes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Desktop widget summary fallback</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>npm.cmd run typecheck; npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Backend summary extended fields are typed and can populate widget display fallback/cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Widget usage rollup retry</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>cd src-tauri; cargo test --lib</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Failed or unmatched usage rollups are marked FAILED in SQLite and remain retry candidates</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Widget window runtime stabilization</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>cd src-tauri; cargo test --lib; npm.cmd run dev:widget:backend; then Windows Tauri GUI smoke</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Windows/non-mac open_widget_window waits for real window creation; existing widgets move with preferred monitor; room context/close-all persist; macOS async build path preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Widget communication voice smoke</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Real backend verifies voice room create/read/mic/leave; token shape is checked when local LiveKit secret allows it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>로컬 파일 분석 서버 왕복</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>/api/local-file-events/sync CREATED returns resourceId, UPDATED preserves it, then /api/local-file-analyses returns ANALYZE_RESOURCE job before DELETE cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>활동 추적 서버 생성/삭제 왕복</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>POST /api/activity/current-app creates a room-scoped record, GET /api/activity/today includes it, DELETE /api/activity/{id} removes it, and /today no longer returns it</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Privacy consent API contract</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>npm.cmd run typecheck; npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Frontend adapter typechecks; smoke asserts GET /api/me/privacy-consents contains ACTIVITY_CONTEXT and MANAGED_FOLDER, PATCH disables/enables MANAGED_FOLDER, then local file sync proceeds with consent re-enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Windows foreground activity capture</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>cargo test --lib</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Windows-only test windows_foreground_capture_returns_app_name calls Win32 foreground capture and asserts non-empty app name</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>SQLite ??</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_db::tests::sqlite_integrity_result_includes_storage_diagnostics; settings cache check in Tauri app</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>quick_check ok plus DB/WAL byte sizes, page count, free page count, and journal mode visible from IPC/UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>?? ?? flush</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run typecheck; npm.cmd run dev:widget:backend; manual Tauri logout/app-close QA</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>On authenticated surface stop, final incremental activity capture and pending buffer sync are attempted before local auto-capture state resets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>??? ???? ??</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend; cargo test --lib local_db::tests::records_and_recovers_running_timer_state</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Start WORK timer in seeded room, dashboard/widget summary expose runningTimer, heartbeat/pause/resume/stop succeed, local recovery test remains green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>Widget item state API</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Seeded TODO task item state changes to PINNED then CONFIRMED through /api/widget/items/{id}/state and PostgreSQL confirms persistence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Widget summary cache account boundary</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>cargo test --lib local_db::tests::widget_summary_cache_is_partitioned_by_cache_key; npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Local widget summary cache stores separate rows per auth subject and real-backend widget smoke still reads current server data successfully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Widget item state item-id fallback</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend against backend branch codex/widget-item-state-upsert-20260703</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>Desktop-widget shaped PATCH using the task item UUID path persists SNOOZED in widget_item_states when no stateId is present in the UI row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Widget item state optimistic UI</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run typecheck; npm.cmd run dev:widget:backend</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>After successful item-state PATCH, desktop widget removes confirmed/hidden/snoozed rows or pins rows locally and keeps the override across the next refresh cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Widget item state readback</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>npm.cmd run dev:widget:backend against backend #183 branch</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>After task-id fallback PATCH persists SNOOZED, GET /api/widget/items/states returns the same state and desktop widget applies persisted states during data load.</t>
         </is>
       </c>
     </row>

</xml_diff>